<commit_message>
Embeber miniaturas de cada producto en el Excel del catálogo
El xlsx ahora abre con una columna "Foto" al inicio que muestra la
primera foto del producto. Felipe ya no necesita abrir las fotos por
separado para saber de cuál hablamos.

- 19 thumbnails generados en branding/assets/productos/thumbs/ (228KB
  total). Rotación EXIF respetada vía PIL.ImageOps.exif_transpose.
- El script reusa thumbs ya generados (idempotente).
- Bug corregido: la primera foto referenciada en algunos productos no
  era la más representativa (posavasos-valdivia mostraba el soporte
  engranaje, cofre-cuadrado-firma mostraba el plegable). Reordenado.
- Layout: freeze pane movido a D4 para que Foto + Categoría + Título
  queden congelados al hacer scroll. Filas de 150pt.
- Hoja Instrucciones actualizada con explicación de la columna Foto.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/branding/catalogo-productos.xlsx
+++ b/branding/catalogo-productos.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Productos'!$A$3:$N$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Productos'!$B$3:$O$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -230,6 +230,486 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1647825"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1647825"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1647825"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1647825"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -521,7 +1001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -550,14 +1030,14 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Columnas en azul claro — propuesta del taller (texto)</t>
+          <t>Columna Foto (A)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Título, bajada, descripción, materialidad, personalización y variantes vienen propuestos por defecto. Si la voz no te calza, edita el texto — la regla está en branding/voz-de-marca.md (registro "taller arquitectónico"): primera persona, frase corta, una idea por frase, cifras y fechas cuando aplique.</t>
+          <t>Cada fila lleva una miniatura de la foto del taller para que sepas a qué producto nos referimos. Si quieres ver la foto original o las demás fotos del producto, mira la columna "Foto referencia" (I).</t>
         </is>
       </c>
     </row>
@@ -567,66 +1047,66 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>Columnas en azul claro — propuesta del taller (texto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Título, bajada, descripción, materialidad, personalización y variantes vienen propuestos por defecto. Si la voz no te calza, edita el texto — la regla está en branding/voz-de-marca.md (registro "taller arquitectónico"): primera persona, frase corta, una idea por frase, cifras y fechas cuando aplique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="10" customHeight="1">
+      <c r="A10" t="inlineStr"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
           <t>Columnas en gris — datos del cliente</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>·  Dimensiones (mm): alto × ancho × profundidad cuando aplique.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>·  Plazo (días): tiempo real de fabricación desde confirmar el pedido.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>·  Precio CLP: precio público B2C. Si tiene variantes, anota el rango (ej. "19.000–29.000").</t>
         </is>
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>·  Foto definitiva: nombre de la foto sobre fondo blanco/Nogal que vamos a usar en la ficha. Por ahora deja vacío o pon "pendiente".</t>
+          <t>·  Dimensiones (mm): alto × ancho × profundidad cuando aplique.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>·  Mostrar en sitio (sí/no): si es "no", queda fuera del catálogo público. Útil para productos que solo se hacen a pedido cerrado.</t>
+          <t>·  Plazo (días): tiempo real de fabricación desde confirmar el pedido.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>·  Precio CLP: precio público B2C. Si tiene variantes, anota el rango (ej. "19.000–29.000").</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>·  Foto definitiva: nombre de la foto sobre fondo blanco/Nogal que vamos a usar en la ficha. Por ahora deja vacío o pon "pendiente".</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>·  Mostrar en sitio (sí/no): si es "no", queda fuera del catálogo público. Útil para productos que solo se hacen a pedido cerrado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>·  Orden: número que define la posición en el listado. 1 = primero. Felipe puede reordenar como quiera; el sitio lo respeta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="10" customHeight="1">
-      <c r="A15" t="inlineStr"/>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Columnas en blanco — solo referencia</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Categoría y Foto referencia son para que sepas de qué producto hablamos. No es necesario editarlas, pero puedes si crees que el producto va en otra categoría.</t>
         </is>
       </c>
     </row>
@@ -636,14 +1116,14 @@
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Cuando termines</t>
+          <t>Columnas en blanco — solo referencia</t>
         </is>
       </c>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Manda este archivo de vuelta. Lo importo a web/maqueta/src/data/products.ts y aparece en lasercrafts.cl con las descripciones que tú aprobaste.</t>
+          <t>Foto (A), Categoría (B) y Foto referencia (I) son para que sepas de qué producto hablamos. No es necesario editarlas, pero puedes si crees que el producto va en otra categoría.</t>
         </is>
       </c>
     </row>
@@ -653,64 +1133,81 @@
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
+          <t>Cuando termines</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Manda este archivo de vuelta. Lo importo a web/maqueta/src/data/products.ts y aparece en lasercrafts.cl con las descripciones que tú aprobaste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="10" customHeight="1">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
           <t>Voz de marca — recordatorio rápido</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>·  Sí: "Lo grabo el martes", "$19.000", "antes del viernes", terciado, taller, Felipe, yo, te.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>·  No: "calidad premium", "plazos competitivos", "nuestro equipo", emojis 🥰💖🎁.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>·  Detalle completo en branding/voz-de-marca.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="10" customHeight="1">
-      <c r="A26" t="inlineStr"/>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>Pendientes generales del catálogo (§13 del .md)</t>
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>·  No: "calidad premium", "plazos competitivos", "nuestro equipo", emojis dulces.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>·  ¿Productos Pokémon/manga se publican o solo a pedido? (IP de terceros)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>·  ¿El cofre porta-posavasos y el cofre cuadrado son uno o dos SKUs distintos?</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="26" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>·  ¿Falta categoría "Matrimonio" (libro de firmas, plano de mesas, distintivos)?</t>
+          <t>·  Detalle completo en branding/voz-de-marca.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="10" customHeight="1">
+      <c r="A29" t="inlineStr"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Pendientes generales del catálogo (§13 del .md)</t>
         </is>
       </c>
     </row>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>·  ¿Productos Pokémon/manga se publican o solo a pedido? (IP de terceros)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>·  ¿El cofre porta-posavasos y el cofre cuadrado son uno o dos SKUs distintos?</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>·  ¿Falta categoría "Matrimonio" (libro de firmas, plano de mesas, distintivos)?</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>·  ¿Falta categoría "Retratos del cliente" (foto grabada en madera)?</t>
         </is>
@@ -727,23 +1224,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
@@ -753,1041 +1251,1066 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="38" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Edita las columnas grises (dimensiones, plazo, precio, foto definitiva, visible, orden). Las columnas azules son la propuesta del taller (título, bajada, descripción) — modifícalas si no calzan con tu voz.</t>
+          <t>Edita las columnas grises (dimensiones, plazo, precio, foto definitiva, visible, orden). Las azules son la propuesta del taller (título, bajada, descripción) — modifícalas si no calzan con tu voz. Detalle de uso y voz de marca en la hoja "Instrucciones".</t>
         </is>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
           <t>Categoría</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Título</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Bajada (lista)</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Descripción (ficha)</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Materialidad</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Personalización</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>Variantes sugeridas</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>Foto referencia</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>Dimensiones (mm)</t>
         </is>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>Plazo (días)</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="L3" s="7" t="inlineStr">
         <is>
           <t>Precio CLP</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr">
+      <c r="M3" s="7" t="inlineStr">
         <is>
           <t>Foto definitiva</t>
         </is>
       </c>
-      <c r="M3" s="7" t="inlineStr">
+      <c r="N3" s="7" t="inlineStr">
         <is>
           <t>Mostrar en sitio (sí/no)</t>
         </is>
       </c>
-      <c r="N3" s="7" t="inlineStr">
+      <c r="O3" s="7" t="inlineStr">
         <is>
           <t>Orden</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="95" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="4" ht="150" customHeight="1">
+      <c r="A4" s="8" t="inlineStr"/>
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Posavasos y mesa</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Posavasos Valdivia</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Posavasos cuadrado en terciado con un pájaro geométrico y la palabra Valdivia.</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>Lo grabamos cuadrado, con un pájaro de líneas geométricas y "Valdivia" en cursiva al lado. Atrás lleva imán, así también sirve de souvenir de refrigerador. Sale solo o en sets de 4 y 6.</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Terciado natural, grabado láser por una cara. Reverso liso con imán.</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>Cambiar la palabra (otra ciudad, un nombre, una fecha).</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>Suelto / Set 4 / Set 6</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>20260328_162735.jpg, 20260328_123630(1).jpg</t>
-        </is>
-      </c>
-      <c r="I4" s="10" t="inlineStr"/>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>20260328_123630(1).jpg, 20260328_123628.jpg</t>
+        </is>
+      </c>
       <c r="J4" s="10" t="inlineStr"/>
       <c r="K4" s="10" t="inlineStr"/>
       <c r="L4" s="10" t="inlineStr"/>
       <c r="M4" s="10" t="inlineStr"/>
-      <c r="N4" s="10" t="n">
+      <c r="N4" s="10" t="inlineStr"/>
+      <c r="O4" s="10" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="5" ht="95" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+    <row r="5" ht="150" customHeight="1">
+      <c r="A5" s="8" t="inlineStr"/>
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Posavasos y mesa</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Posavasos fauna nativa</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Posavasos redondos con grabado de fauna nativa y su nombre científico.</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Cada pieza es una especie del sur de Chile, grabada en línea fina con nombre común y científico al borde. Hoy hemos hecho cisne cuello negro, martín pescador y otras aves del bosque valdiviano. Se piden por especie o como set temático (parques, viñas, hoteles).</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>Terciado, grabado por una cara, sin pintar.</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Elegir especies, agregar logo institucional al reverso.</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>Cisne cuello negro / Martín pescador / a definir</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>20260531_135930.jpg, 20260531_140635.jpg</t>
         </is>
       </c>
-      <c r="I5" s="10" t="inlineStr"/>
       <c r="J5" s="10" t="inlineStr"/>
       <c r="K5" s="10" t="inlineStr"/>
       <c r="L5" s="10" t="inlineStr"/>
       <c r="M5" s="10" t="inlineStr"/>
-      <c r="N5" s="10" t="n">
+      <c r="N5" s="10" t="inlineStr"/>
+      <c r="O5" s="10" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="6" ht="95" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="6" ht="150" customHeight="1">
+      <c r="A6" s="8" t="inlineStr"/>
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Posavasos y mesa</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Set posavasos geométricos + cofre</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Cuatro posavasos calados con patrones geométricos, presentados en cofre con la firma LáserCrafts.</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Cuatro patrones distintos —asanoha, seigaiha y dos más— calados en terciado, listos para servir en mesa de café. Vienen en un cofre cuadrado con la firma del taller grabada al fondo. Es nuestro regalo corporativo más pedido.</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Terciado, calado pasante, sin pintar.</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Grabado en la tapa o el frente del cofre con el logo o nombre del cliente.</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>Set 4 patrones (estándar) / personalizado</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>20260328_122332.jpg, 20260328_122324.jpg</t>
         </is>
       </c>
-      <c r="I6" s="10" t="inlineStr"/>
       <c r="J6" s="10" t="inlineStr"/>
       <c r="K6" s="10" t="inlineStr"/>
       <c r="L6" s="10" t="inlineStr"/>
       <c r="M6" s="10" t="inlineStr"/>
-      <c r="N6" s="10" t="n">
+      <c r="N6" s="10" t="inlineStr"/>
+      <c r="O6" s="10" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="7" ht="95" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="7" ht="150" customHeight="1">
+      <c r="A7" s="8" t="inlineStr"/>
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Posavasos y mesa</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Bandeja porta-posavasos</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Bandeja baja con la firma LáserCrafts grabada al frente, lista para una mesa de café.</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>La bandeja sostiene seis posavasos y una taza al medio. La grabamos al frente con el nombre de quien la regala o la marca del local que la pide. Cabe en mesa de centro o repisa de cocina.</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>MDF con grabado láser por una cara.</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Texto al frente (nombre, marca, frase).</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>Estándar / personalizado</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>20260328_115416.jpg</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="10" t="inlineStr"/>
       <c r="K7" s="10" t="inlineStr"/>
       <c r="L7" s="10" t="inlineStr"/>
       <c r="M7" s="10" t="inlineStr"/>
-      <c r="N7" s="10" t="n">
+      <c r="N7" s="10" t="inlineStr"/>
+      <c r="O7" s="10" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="8" ht="95" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="8" ht="150" customHeight="1">
+      <c r="A8" s="8" t="inlineStr"/>
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Cofres y cajas</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Cofre tapa de hojas</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Cofre rectangular con tapa de hojas caladas, para guardar lo que sea importante.</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>La tapa es una composición de hojas caladas que se cruzan; la luz pasa entre ellas. Adentro cabe joyería, un anillo de matrimonio, recuerdos. Es el cofre que más pedimos para nacimientos y aniversarios.</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>Terciado, calado pasante en la tapa, cuerpo cerrado.</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>Grabado interior (nombre, fecha) en el fondo de la caja.</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>Estándar / con grabado interior</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>20260328_110045.jpg, 20260328_110159.jpg</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="10" t="inlineStr"/>
       <c r="K8" s="10" t="inlineStr"/>
       <c r="L8" s="10" t="inlineStr"/>
       <c r="M8" s="10" t="inlineStr"/>
-      <c r="N8" s="10" t="n">
+      <c r="N8" s="10" t="inlineStr"/>
+      <c r="O8" s="10" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="9" ht="95" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="9" ht="150" customHeight="1">
+      <c r="A9" s="8" t="inlineStr"/>
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Cofres y cajas</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Cofre cuadrado firma LáserCrafts</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Cofre cuadrado con la firma del taller grabada al fondo.</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>Lo armamos a la medida del set de posavasos, pero también funciona como cofre solo. La firma queda escondida al fondo, así el cliente la descubre al abrir.</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Terciado, grabado al fondo.</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>Mensaje grabado al fondo (sustituye la firma) o en la tapa.</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="H9" s="9" t="inlineStr">
         <is>
           <t>Solo / con set de posavasos</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>20260328_122332.jpg, 20260328_123021.jpg</t>
-        </is>
-      </c>
-      <c r="I9" s="10" t="inlineStr"/>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>20260328_122332.jpg, 20260328_122324.jpg</t>
+        </is>
+      </c>
       <c r="J9" s="10" t="inlineStr"/>
       <c r="K9" s="10" t="inlineStr"/>
       <c r="L9" s="10" t="inlineStr"/>
       <c r="M9" s="10" t="inlineStr"/>
-      <c r="N9" s="10" t="n">
+      <c r="N9" s="10" t="inlineStr"/>
+      <c r="O9" s="10" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="10" ht="95" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="10" ht="150" customHeight="1">
+      <c r="A10" s="8" t="inlineStr"/>
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Soportes para escritorio</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Soporte de celular plegable</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Soporte de celular que se pliega, con grabado al frente.</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>Lo grabamos con el logo de un equipo, una marca o una frase. Se pliega cuando no se usa y queda como pieza de escritorio. Sirve para celular y para tablet pequeña.</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>MDF, grabado láser al frente.</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>Grabado al frente (escudo de equipo, logo, frase, nombre).</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="H10" s="9" t="inlineStr">
         <is>
           <t>Logo personalizado / estándar</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>20260328_123021.jpg</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="10" t="inlineStr"/>
       <c r="K10" s="10" t="inlineStr"/>
       <c r="L10" s="10" t="inlineStr"/>
       <c r="M10" s="10" t="inlineStr"/>
-      <c r="N10" s="10" t="n">
+      <c r="N10" s="10" t="inlineStr"/>
+      <c r="O10" s="10" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="11" ht="95" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="11" ht="150" customHeight="1">
+      <c r="A11" s="8" t="inlineStr"/>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Soportes para escritorio</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>Soporte de celular engranaje</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Soporte para celular con engranaje calado y madera oscura.</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>El detalle del engranaje queda visible al apoyar el celular. Lo entregamos en madera oscura para que el contraste con el grabado sea fuerte. Es nuestro soporte más vendido a personas que trabajan en escritorio.</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>MDF teñido oscuro, calado y armado por encastre.</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>Grabado al lateral del engranaje.</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>Estándar / con grabado lateral</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>20260328_162735.jpg</t>
         </is>
       </c>
-      <c r="I11" s="10" t="inlineStr"/>
       <c r="J11" s="10" t="inlineStr"/>
       <c r="K11" s="10" t="inlineStr"/>
       <c r="L11" s="10" t="inlineStr"/>
       <c r="M11" s="10" t="inlineStr"/>
-      <c r="N11" s="10" t="n">
+      <c r="N11" s="10" t="inlineStr"/>
+      <c r="O11" s="10" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="12" ht="150" customHeight="1">
+      <c r="A12" s="8" t="inlineStr"/>
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Pins, imanes y llaveros</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Set pins/imanes naturaleza</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Set de cuatro pins pintados a mano: hongo amanita, pino con luna, hongo violeta, mariposa luna.</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>Cada pieza la pintamos a mano sobre el grabado, así no hay dos exactamente iguales. Se piden sueltos o en sets de cuatro. Se usan como pin de mochila, imán de refrigerador o adorno de planta.</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>Terciado o MDF, grabado láser, pintado a mano.</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>Elegir las cuatro piezas del set entre las disponibles.</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="H12" s="9" t="inlineStr">
         <is>
           <t>Suelto / Set 4</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="I12" s="8" t="inlineStr">
         <is>
           <t>20260328_111352.jpg, 20260328_111414.jpg, 20260328_111253.jpg</t>
         </is>
       </c>
-      <c r="I12" s="10" t="inlineStr"/>
       <c r="J12" s="10" t="inlineStr"/>
       <c r="K12" s="10" t="inlineStr"/>
       <c r="L12" s="10" t="inlineStr"/>
       <c r="M12" s="10" t="inlineStr"/>
-      <c r="N12" s="10" t="n">
+      <c r="N12" s="10" t="inlineStr"/>
+      <c r="O12" s="10" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="13" ht="95" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="13" ht="150" customHeight="1">
+      <c r="A13" s="8" t="inlineStr"/>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Pins, imanes y llaveros</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>Llaveros fauna nativa</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Llaveros de pájaros y mamíferos del bosque valdiviano, con nombre al lado.</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>Hoy tenemos chucao y monito del monte; vamos sumando especies según pedidos. El reverso queda limpio para grabar el logo de quien los regala (parque, hotel, viña). Llevan anilla metálica y cadena corta.</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>Terciado, grabado láser por las dos caras, anilla metálica.</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>Logo institucional al reverso, set por temática (aves, mamíferos, hongos).</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>Chucao / Monito del monte / + a definir</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>20260531_130739.jpg, 20260531_131826.jpg, 20260531_131635.jpg</t>
         </is>
       </c>
-      <c r="I13" s="10" t="inlineStr"/>
       <c r="J13" s="10" t="inlineStr"/>
       <c r="K13" s="10" t="inlineStr"/>
       <c r="L13" s="10" t="inlineStr"/>
       <c r="M13" s="10" t="inlineStr"/>
-      <c r="N13" s="10" t="n">
+      <c r="N13" s="10" t="inlineStr"/>
+      <c r="O13" s="10" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="14" ht="95" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="14" ht="150" customHeight="1">
+      <c r="A14" s="8" t="inlineStr"/>
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Marcapáginas</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>Marcapáginas fauna nativa</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Marcapáginas en terciado con flora y hongos del sur, nombre común y científico.</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>La forma sigue al organismo —el digüeñe es una cabeza de racimos, el campañita magallánica es un hongo entero con su raíz, otros son árboles con copa y raíz. En el cabezal va el nombre común y el científico abajo. Pensados para librería independiente, museo o regalo botánico.</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>Terciado, grabado por una cara, contorno calado.</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="G14" s="9" t="inlineStr">
         <is>
           <t>Elegir las especies del set, agregar logo en el cabezal.</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>Digüeñe / Campañita magallánica / + a definir</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>20260531_125703.jpg, 20260531_130023.jpg, 20260531_130419.jpg</t>
-        </is>
-      </c>
-      <c r="I14" s="10" t="inlineStr"/>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>20260531_130023.jpg, 20260531_125703.jpg, 20260531_130419.jpg</t>
+        </is>
+      </c>
       <c r="J14" s="10" t="inlineStr"/>
       <c r="K14" s="10" t="inlineStr"/>
       <c r="L14" s="10" t="inlineStr"/>
       <c r="M14" s="10" t="inlineStr"/>
-      <c r="N14" s="10" t="n">
+      <c r="N14" s="10" t="inlineStr"/>
+      <c r="O14" s="10" t="n">
         <v>11</v>
       </c>
     </row>
-    <row r="15" ht="95" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="15" ht="150" customHeight="1">
+      <c r="A15" s="8" t="inlineStr"/>
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Cuadros 3D multicapa</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>Cuadro 3D pez betta</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Cuadro enmarcado con un pez betta en relieve sobre fondo de peces grabados.</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>El pez se arma en varias capas de madera teñida, así sus aletas tienen profundidad real (no es solo grabado). El fondo es una trama de peces más pequeños grabados en plano. Marco oscuro, listo para colgar.</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>Terciado multicapa, teñido, marco oscuro.</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>Elegir tonos del pez (rojo, azul, dorado).</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t>Rojo / Azul / Dorado</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
+      <c r="I15" s="8" t="inlineStr">
         <is>
           <t>20260328_111942.jpg</t>
         </is>
       </c>
-      <c r="I15" s="10" t="inlineStr"/>
       <c r="J15" s="10" t="inlineStr"/>
       <c r="K15" s="10" t="inlineStr"/>
       <c r="L15" s="10" t="inlineStr"/>
       <c r="M15" s="10" t="inlineStr"/>
-      <c r="N15" s="10" t="n">
+      <c r="N15" s="10" t="inlineStr"/>
+      <c r="O15" s="10" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="16" ht="95" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="16" ht="150" customHeight="1">
+      <c r="A16" s="8" t="inlineStr"/>
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Cuadros 3D multicapa</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>Cuadro 3D personaje manga/anime</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Retrato 3D armado en capas: personaje sobre fondo decorativo, marco listo para colgar.</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>Lo hacemos a pedido sobre un personaje que mande el cliente. Se arma en cuatro a seis capas, con colores planos en rojo, azul, gris y negro. Llega con bastidor, listo para colgar.</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>Terciado multicapa, teñido a mano, montado en bastidor.</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
         <is>
           <t>A medida — el cliente manda el personaje o la imagen base.</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>A medida</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="I16" s="8" t="inlineStr">
         <is>
           <t>20260328_113614.jpg</t>
         </is>
       </c>
-      <c r="I16" s="10" t="inlineStr"/>
       <c r="J16" s="10" t="inlineStr"/>
       <c r="K16" s="10" t="inlineStr"/>
       <c r="L16" s="10" t="inlineStr"/>
       <c r="M16" s="10" t="inlineStr"/>
-      <c r="N16" s="10" t="n">
+      <c r="N16" s="10" t="inlineStr"/>
+      <c r="O16" s="10" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="17" ht="95" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="17" ht="150" customHeight="1">
+      <c r="A17" s="8" t="inlineStr"/>
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Coleccionables Pokémon</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>Carta Pokémon 3D</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Reproducción 3D de carta Pokémon armada en capas y pintada a mano.</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>El holograma de la carta se reemplaza por capas de madera grabadas y pintadas: el Pokémon en relieve, el fondo, el contorno y el texto. Cada una toma tiempo, así que las hacemos a pedido. Hoy hemos hecho Leafeon Vmax, Pikachu y Wartortle, pero se puede pedir otra.</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>Terciado multicapa, grabado y pintado a mano.</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>A medida — el cliente elige el Pokémon, la carta y los colores.</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="H17" s="9" t="inlineStr">
         <is>
           <t>Leafeon Vmax / Pikachu / Wartortle / + a pedido</t>
         </is>
       </c>
-      <c r="H17" s="8" t="inlineStr">
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>20260328_123148.jpg, 20260328_123132.jpg, 20260328_122951.jpg</t>
         </is>
       </c>
-      <c r="I17" s="10" t="inlineStr"/>
       <c r="J17" s="10" t="inlineStr"/>
       <c r="K17" s="10" t="inlineStr"/>
       <c r="L17" s="10" t="inlineStr"/>
       <c r="M17" s="10" t="inlineStr"/>
-      <c r="N17" s="10" t="n">
+      <c r="N17" s="10" t="inlineStr"/>
+      <c r="O17" s="10" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="18" ht="95" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="18" ht="150" customHeight="1">
+      <c r="A18" s="8" t="inlineStr"/>
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Coleccionables Pokémon</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>Set medallas de gimnasio</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Set de seis medallas de gimnasio pintadas a mano.</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>Reproducimos las medallas clásicas: roca, agua, fuego, hoja, espina, planta, alma y otras. Se piden por unidad o como set completo, atrás llevan imán. Es regalo cumpleaños fan #1 del año.</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>MDF, grabado, pintado a mano, imán al reverso.</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
         <is>
           <t>Elegir qué medallas entran en el set.</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>Suelto / Set 6 / Set 8</t>
         </is>
       </c>
-      <c r="H18" s="8" t="inlineStr">
+      <c r="I18" s="8" t="inlineStr">
         <is>
           <t>20260328_111549.jpg</t>
         </is>
       </c>
-      <c r="I18" s="10" t="inlineStr"/>
       <c r="J18" s="10" t="inlineStr"/>
       <c r="K18" s="10" t="inlineStr"/>
       <c r="L18" s="10" t="inlineStr"/>
       <c r="M18" s="10" t="inlineStr"/>
-      <c r="N18" s="10" t="n">
+      <c r="N18" s="10" t="inlineStr"/>
+      <c r="O18" s="10" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="19" ht="95" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+    <row r="19" ht="150" customHeight="1">
+      <c r="A19" s="8" t="inlineStr"/>
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Casitas armables y maquetas</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>Casa Halloween armable</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>Casa fantasma armable en madera, con espacio para vela LED y figuras alrededor.</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>Llega plana, se arma por encastre. Lleva fachada con telarañas grabadas, ventanas troqueladas, calabaza al frente, fantasma colgando y carteles de "Ghost Crossing" y "Witches Way". El espacio interior recibe una vela LED para que las ventanas brillen.</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>MDF, pintado a mano, encastre.</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
         <is>
           <t>Nombre del niño/a en el frente, año de la fiesta.</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t>Estándar / personalizada</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>20260328_114526.jpg</t>
         </is>
       </c>
-      <c r="I19" s="10" t="inlineStr"/>
       <c r="J19" s="10" t="inlineStr"/>
       <c r="K19" s="10" t="inlineStr"/>
       <c r="L19" s="10" t="inlineStr"/>
       <c r="M19" s="10" t="inlineStr"/>
-      <c r="N19" s="10" t="n">
+      <c r="N19" s="10" t="inlineStr"/>
+      <c r="O19" s="10" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="20" ht="95" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
+    <row r="20" ht="150" customHeight="1">
+      <c r="A20" s="8" t="inlineStr"/>
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Placas y letreros</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Placa de dirección con escena</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>Placa para la entrada con número de calle y una escena grabada del lugar.</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>El cliente manda foto de su casa, dibujo o referencia; nosotros la traducimos a grabado. Va con el número de calle grabado grande y la escena al lado. Se cuelga afuera o en el living como recuerdo del lugar.</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>Terciado, grabado por una cara, perforaciones para colgar.</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="G20" s="9" t="inlineStr">
         <is>
           <t>A medida — el dibujo, el número, el nombre de la familia.</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="H20" s="9" t="inlineStr">
         <is>
           <t>A medida</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="I20" s="8" t="inlineStr">
         <is>
           <t>20260328_120002.jpg</t>
         </is>
       </c>
-      <c r="I20" s="10" t="inlineStr"/>
       <c r="J20" s="10" t="inlineStr"/>
       <c r="K20" s="10" t="inlineStr"/>
       <c r="L20" s="10" t="inlineStr"/>
       <c r="M20" s="10" t="inlineStr"/>
-      <c r="N20" s="10" t="n">
+      <c r="N20" s="10" t="inlineStr"/>
+      <c r="O20" s="10" t="n">
         <v>17</v>
       </c>
     </row>
-    <row r="21" ht="95" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="21" ht="150" customHeight="1">
+      <c r="A21" s="8" t="inlineStr"/>
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Placas y letreros</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>Letrero exterior para tienda</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Letrero colgante en madera con grabado del logo y tagline de la marca.</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>Lo hacemos para comercios pequeños que quieren un cartel exterior que no parezca impreso. Trabajamos con vectorial del cliente o lo redibujamos juntos. Va terminado con barniz exterior y herrajes para colgar.</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Terciado o tablón, grabado, pintado, barniz exterior, herraje de hierro.</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t>A medida — el logo, los colores, las dimensiones.</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t>A medida</t>
         </is>
       </c>
-      <c r="H21" s="8" t="inlineStr">
+      <c r="I21" s="8" t="inlineStr">
         <is>
           <t>20260328_115809.jpg</t>
         </is>
       </c>
-      <c r="I21" s="10" t="inlineStr"/>
       <c r="J21" s="10" t="inlineStr"/>
       <c r="K21" s="10" t="inlineStr"/>
       <c r="L21" s="10" t="inlineStr"/>
       <c r="M21" s="10" t="inlineStr"/>
-      <c r="N21" s="10" t="n">
+      <c r="N21" s="10" t="inlineStr"/>
+      <c r="O21" s="10" t="n">
         <v>18</v>
       </c>
     </row>
-    <row r="22" ht="95" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+    <row r="22" ht="150" customHeight="1">
+      <c r="A22" s="8" t="inlineStr"/>
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Encargos a medida</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Expositor Hot Wheels</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Expositor mural en MDF para colección de Hot Wheels con logo grabado.</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>Lo armamos para coleccionistas serios: tres columnas, soportes para que las cajas queden inclinadas y visibles, logo Hot Wheels grabado al frente. Cabe en muro y se llena de a poco.</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>MDF teñido oscuro, grabado, herraje para muro.</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
         <is>
           <t>A medida — cantidad de columnas, tipo de colección (Pokémon, Funko, Tarot, etc.).</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="H22" s="9" t="inlineStr">
         <is>
           <t>A medida</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr">
+      <c r="I22" s="8" t="inlineStr">
         <is>
           <t>IMG-20260328-WA0058.jpg</t>
         </is>
       </c>
-      <c r="I22" s="10" t="inlineStr"/>
       <c r="J22" s="10" t="inlineStr"/>
       <c r="K22" s="10" t="inlineStr"/>
       <c r="L22" s="10" t="inlineStr"/>
       <c r="M22" s="10" t="inlineStr"/>
-      <c r="N22" s="10" t="n">
+      <c r="N22" s="10" t="inlineStr"/>
+      <c r="O22" s="10" t="n">
         <v>19</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N22"/>
+  <autoFilter ref="B3:O22"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:O2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Recortar fondo de las 19 fotos de productos con rembg
Las fotos del taller venían sobre el "studio box" de cartón con
patrones punteados al fondo. Procesadas con rembg (modelo neural
u2net) para dejar solo el producto sobre fondo blanco puro.

- branding/assets/scripts/clean-product-photos.py: pipeline
  reproducible (EXIF → rembg → composición sobre blanco → crop al
  bounding box con 6% padding → resize). Idempotente, --force para
  regenerar.
- branding/assets/productos/thumbs/: thumbs 280px regenerados (para
  el Excel del cliente).
- web/maqueta/public/img/products/catalogo/: imágenes 900px de ancho
  para las fichas y listados del sitio.
- catalogo-productos.xlsx regenerado con los thumbs limpios.
- Sitio rebuild (37 páginas) — los productos en /productos/ y las
  fichas /producto/<slug>/ ahora muestran las fotos limpias.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/branding/catalogo-productos.xlsx
+++ b/branding/catalogo-productos.xlsx
@@ -241,7 +241,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1238250" cy="581025"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -266,7 +266,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1647825"/>
+    <ext cx="1238250" cy="1181100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -291,7 +291,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1238250" cy="933450"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -316,7 +316,7 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1238250" cy="495300"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -341,7 +341,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="952500" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -366,7 +366,7 @@
       <row>8</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1238250" cy="933450"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -391,7 +391,7 @@
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1152525" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
@@ -416,7 +416,7 @@
       <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1123950" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="8" name="Image 8" descr="Picture"/>
@@ -441,7 +441,7 @@
       <row>11</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1238250" cy="447675"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -466,7 +466,7 @@
       <row>12</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1647825"/>
+    <ext cx="1238250" cy="1447800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -491,7 +491,7 @@
       <row>13</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1647825"/>
+    <ext cx="1238250" cy="1133475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -516,7 +516,7 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1238250" cy="1590675"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>
@@ -541,7 +541,7 @@
       <row>15</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1123950" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="13" name="Image 13" descr="Picture"/>
@@ -566,7 +566,7 @@
       <row>16</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1038225" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="14" name="Image 14" descr="Picture"/>
@@ -591,7 +591,7 @@
       <row>17</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1238250" cy="523875"/>
     <pic>
       <nvPicPr>
         <cNvPr id="15" name="Image 15" descr="Picture"/>
@@ -616,7 +616,7 @@
       <row>18</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1219200" cy="1714500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="16" name="Image 16" descr="Picture"/>
@@ -641,7 +641,7 @@
       <row>19</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1238250" cy="1019175"/>
     <pic>
       <nvPicPr>
         <cNvPr id="17" name="Image 17" descr="Picture"/>
@@ -666,7 +666,7 @@
       <row>20</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1238250"/>
+    <ext cx="1238250" cy="1362075"/>
     <pic>
       <nvPicPr>
         <cNvPr id="18" name="Image 18" descr="Picture"/>

</xml_diff>

<commit_message>
Fotos de productos cuadradas con margen blanco generoso
Las imágenes de catálogo ahora son cuadradas (1:1) con 18% de margen
blanco a cada lado del producto. Resultado: grilla uniforme y producto
"respirado" en cada card.

- clean-product-photos.py: después de rembg y crop al bounding box,
  se compone sobre canvas cuadrado blanco con lado =
  max(producto_w, producto_h) * 1.36. Producto centrado.
- ROTATE_OVERRIDES vacío por ahora (la orientación que entrega rembg
  es la correcta para todos los productos del primer lote).
- Excel regenerado con thumbs cuadrados.
- Sitio rebuild — /productos y /producto/<slug> ahora muestran cards
  perfectamente alineadas.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/branding/catalogo-productos.xlsx
+++ b/branding/catalogo-productos.xlsx
@@ -241,7 +241,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="581025"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -266,7 +266,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1181100"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -291,7 +291,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="933450"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -316,7 +316,7 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="495300"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -341,7 +341,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="952500" cy="1714500"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -366,7 +366,7 @@
       <row>8</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="933450"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -391,7 +391,7 @@
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1152525" cy="1714500"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
@@ -416,7 +416,7 @@
       <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1123950" cy="1714500"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="8" name="Image 8" descr="Picture"/>
@@ -441,7 +441,7 @@
       <row>11</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="447675"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -466,7 +466,7 @@
       <row>12</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1447800"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -491,7 +491,7 @@
       <row>13</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1133475"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -516,7 +516,7 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1590675"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>
@@ -541,7 +541,7 @@
       <row>15</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1123950" cy="1714500"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="13" name="Image 13" descr="Picture"/>
@@ -566,7 +566,7 @@
       <row>16</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1038225" cy="1714500"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="14" name="Image 14" descr="Picture"/>
@@ -591,7 +591,7 @@
       <row>17</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="523875"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="15" name="Image 15" descr="Picture"/>
@@ -616,7 +616,7 @@
       <row>18</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1219200" cy="1714500"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="16" name="Image 16" descr="Picture"/>
@@ -641,7 +641,7 @@
       <row>19</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1019175"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="17" name="Image 17" descr="Picture"/>
@@ -666,7 +666,7 @@
       <row>20</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1362075"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="18" name="Image 18" descr="Picture"/>
@@ -691,7 +691,7 @@
       <row>21</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1238250" cy="1647825"/>
+    <ext cx="1238250" cy="1238250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="19" name="Image 19" descr="Picture"/>

</xml_diff>